<commit_message>
Små oppdateringer litt her og der
</commit_message>
<xml_diff>
--- a/reports/hazop_system_24.xlsx
+++ b/reports/hazop_system_24.xlsx
@@ -8,7 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="24-PA001-section" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="loop 24-001" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="loop 24-2001" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="loop 24-2100" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="loop 24-2159" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="loop 24-2160" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="loop 24-2162" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="loop 24-2163" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -464,7 +470,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HAZOP preparation — System 24 (DEXPI process sections)</t>
+          <t>HAZOP preparation — System 24 (functional loops)</t>
         </is>
       </c>
     </row>
@@ -508,22 +514,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>24-PA001-section</t>
+          <t>loop 24-001</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>24-2007PL, 24-2008PL, 24-2009PL, 24-2010PL, 24-2052PL, 24-2053PL, 24-2054PL, 24-2055PL, 24-2056PL, 24-2057PL, 24-2059PL, 24-2060PL, 24-2061PL, 24-FIC2100, 24-FT2100, 24-FV2100, 24-FY2100, 24-LSH2005, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-PA001, 24-PDI2001, 24-PI2159, 24-PI2160, 24-PT2159, 24-PT2160, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B, 56-2003PL, 57-2001PL</t>
+          <t>24-PA001, 24-PE001</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -532,8 +538,170 @@
         <v>0</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>loop 24-2001</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>24-PDI2001, 24-PI2001, 24-PT2001</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>loop 24-2100</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>24-FIC2100, 24-FT2100, 24-FV2100, 24-FY2100</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>loop 24-2159</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>24-PI2159, 24-PT2159</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>loop 24-2160</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>24-PI2160, 24-PT2160</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>loop 24-2162</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>24-LIC2162, 24-LIC2162A, 24-LIC2162B, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>loop 24-2163</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-XY2163A, 24-XY2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>AI-prepared draft from extracted P&amp;ID/SCD data — for HAZOP team review, not a completed study.</t>
         </is>
@@ -550,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -568,14 +736,14 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Node: 24-PA001-section</t>
+          <t>Node: loop 24-001</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Members: 24-2007PL, 24-2008PL, 24-2009PL, 24-2010PL, 24-2052PL, 24-2053PL, 24-2054PL, 24-2055PL, 24-2056PL, 24-2057PL, 24-2059PL, 24-2060PL, 24-2061PL, 24-FIC2100, 24-FT2100, 24-FV2100, 24-FY2100, 24-LSH2005, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-PA001, 24-PDI2001, 24-PI2159, 24-PI2160, 24-PT2159, 24-PT2160, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B, 56-2003PL, 57-2001PL</t>
+          <t>Members: 24-PA001, 24-PE001</t>
         </is>
       </c>
     </row>
@@ -634,22 +802,22 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>No flow</t>
+          <t>High pressure</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>24-FIC2100: wrong output; 24-FIC2100: tuning drift; 24-FV2100: sticks; 24-FV2100: wrong position; blocked line / closed valve (generic); pump/compressor stop (generic)</t>
+          <t>blocked outlet (generic); upstream pressure source (generic)</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>loss of process function (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-XV2163A, 24-XV2163B; safety functions in node: 24-LSH2005, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+          <t>possible overpressure of section (generic)</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
+          <t>(none found in extraction — verify)</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr"/>
@@ -666,22 +834,22 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Low flow</t>
+          <t>Low pressure</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>24-FIC2100: wrong output; 24-FIC2100: tuning drift; 24-FV2100: sticks; 24-FV2100: wrong position; partial blockage / fouling (generic)</t>
+          <t>upstream supply loss (generic); leak / rupture (generic)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>reduced capacity (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-XV2163A, 24-XV2163B; safety functions in node: 24-LSH2005, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+          <t>loss of process function / possible gas breakthrough (generic)</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
+          <t>(none found in extraction — verify)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr"/>
@@ -695,6 +863,318 @@
         </is>
       </c>
     </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Node: loop 24-2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Members: 24-PDI2001, 24-PI2001, 24-PT2001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Deviation</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Causes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Consequences</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Safeguards</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Action party</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>High pressure</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>blocked outlet (generic); upstream pressure source (generic)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>possible overpressure of section (generic)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Low pressure</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>upstream supply loss (generic); leak / rupture (generic)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>loss of process function / possible gas breakthrough (generic)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Node: loop 24-2100</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Members: 24-FIC2100, 24-FT2100, 24-FV2100, 24-FY2100</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Deviation</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Causes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Consequences</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Safeguards</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Action party</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>No flow</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>24-FIC2100: wrong output; 24-FIC2100: tuning drift; 24-FV2100: sticks; 24-FV2100: wrong position; blocked line / closed valve (generic); pump/compressor stop (generic)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>loss of process function (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Low flow</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>24-FIC2100: wrong output; 24-FIC2100: tuning drift; 24-FV2100: sticks; 24-FV2100: wrong position; partial blockage / fouling (generic)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>reduced capacity (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -708,12 +1188,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>possible downstream overload (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-XV2163A, 24-XV2163B; safety functions in node: 24-LSH2005, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+          <t>possible downstream overload (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
+          <t>(none found in extraction — verify)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr"/>
@@ -740,12 +1220,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>possible contamination / backflow to upstream (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-XV2163A, 24-XV2163B; safety functions in node: 24-LSH2005, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+          <t>possible contamination / backflow to upstream (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
+          <t>(none found in extraction — verify)</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr"/>
@@ -759,129 +1239,689 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Node: loop 24-2159</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Members: 24-PI2159, 24-PT2159</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Deviation</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Causes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Consequences</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Safeguards</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Action party</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>High pressure</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>blocked outlet (generic); upstream pressure source (generic)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>possible overpressure of section (generic)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Low pressure</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>upstream supply loss (generic); leak / rupture (generic)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>loss of process function / possible gas breakthrough (generic)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Node: loop 24-2160</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Members: 24-PI2160, 24-PT2160</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Deviation</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Causes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Consequences</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Safeguards</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Action party</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>High pressure</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>blocked outlet (generic); upstream pressure source (generic)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>possible overpressure of section (generic)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Low pressure</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>upstream supply loss (generic); leak / rupture (generic)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>loss of process function / possible gas breakthrough (generic)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Node: loop 24-2162</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Members: 24-LIC2162, 24-LIC2162A, 24-LIC2162B, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Deviation</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Causes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Consequences</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Safeguards</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Action party</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>High level</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>24-FIC2100: wrong output; 24-FIC2100: tuning drift; 24-FV2100: sticks; 24-FV2100: wrong position; outlet restriction (generic); inflow exceeds outflow (generic)</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>possible carry-over / overfill (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-XV2163A, 24-XV2163B; safety functions in node: 24-LSH2005, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>24-LSH2005 (⚠ same loop — verify independence), 24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr"/>
-      <c r="H8" s="6" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>24-LIC2162: wrong output; 24-LIC2162: tuning drift; 24-LIC2162A: wrong output; 24-LIC2162A: tuning drift; 24-LIC2162B: wrong output; 24-LIC2162B: tuning drift; outlet restriction (generic); inflow exceeds outflow (generic)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>possible carry-over / overfill (generic); functions affected: 24-LIC2162, 24-LIC2162A, 24-LIC2162B, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Low level</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>24-FIC2100: wrong output; 24-FIC2100: tuning drift; 24-FV2100: sticks; 24-FV2100: wrong position; loss of feed (generic); excess drainage (generic)</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>possible gas blow-by to downstream (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-XV2163A, 24-XV2163B; safety functions in node: 24-LSH2005, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>24-LIC2162: wrong output; 24-LIC2162: tuning drift; 24-LIC2162A: wrong output; 24-LIC2162A: tuning drift; 24-LIC2162B: wrong output; 24-LIC2162B: tuning drift; loss of feed (generic); excess drainage (generic)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>possible gas blow-by to downstream (generic); functions affected: 24-LIC2162, 24-LIC2162A, 24-LIC2162B, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>(none found in extraction — verify)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Node: loop 24-2163</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Members: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-XY2163A, 24-XY2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Deviation</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Causes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Consequences</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Safeguards</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Action party</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>No flow</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>blocked line / closed valve (generic); pump/compressor stop (generic)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>loss of process function (generic); functions affected: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-XY2163A, 24-XY2163B; safety functions in node: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>High pressure</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>24-FIC2100: wrong output; 24-FIC2100: tuning drift; 24-FV2100: sticks; 24-FV2100: wrong position; blocked outlet (generic); upstream pressure source (generic)</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>possible overpressure of section (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-XV2163A, 24-XV2163B; safety functions in node: 24-LSH2005, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Low flow</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>partial blockage / fouling (generic)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>reduced capacity (generic); functions affected: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-XY2163A, 24-XY2163B; safety functions in node: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="6" t="inlineStr"/>
-      <c r="I10" s="6" t="inlineStr"/>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Low pressure</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>24-FIC2100: wrong output; 24-FIC2100: tuning drift; 24-FV2100: sticks; 24-FV2100: wrong position; upstream supply loss (generic); leak / rupture (generic)</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>loss of process function / possible gas breakthrough (generic); functions affected: 24-FIC2100, 24-FV2100, 24-FY2100, 24-LV2162A, 24-LV2162B, 24-LY2162A, 24-LY2162B, 24-XV2163A, 24-XV2163B; safety functions in node: 24-LSH2005, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>High flow</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>control valve fully open (generic)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>possible downstream overload (generic); functions affected: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-XY2163A, 24-XY2163B; safety functions in node: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="6" t="inlineStr"/>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="6" t="inlineStr"/>
-      <c r="I11" s="6" t="inlineStr"/>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Reverse flow</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>check-valve failure / pressure reversal (generic)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>possible contamination / backflow to upstream (generic); functions affected: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-XY2163A, 24-XY2163B; safety functions in node: 24-HS2163, 24-HS2163A, 24-HS2163B, 24-XV2163A, 24-XV2163B, 24-ZL2163A, 24-ZL2163B, 24-ZS2163A, 24-ZS2163B</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>24-XV2163A (⚠ same loop — verify independence), 24-XV2163B (⚠ same loop — verify independence)</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>

</xml_diff>